<commit_message>
Login and Download features developed
</commit_message>
<xml_diff>
--- a/GPO Roster Avendra/Data/Config.xlsx
+++ b/GPO Roster Avendra/Data/Config.xlsx
@@ -1,28 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubAnkush\GPO-Roster-Hilton\GPO Roster Hilton\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubSai\GPO-Roster-Avendra\GPO Roster Avendra\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70AB830-A8F2-4409-B9A9-1D55189E663B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7816604-42F4-405C-B7EC-4E8170D4FC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="85">
   <si>
     <t>Name</t>
   </si>
@@ -162,15 +175,6 @@
     <t>ProcessABCQueue</t>
   </si>
   <si>
-    <t>HSM_URL</t>
-  </si>
-  <si>
-    <t>https://hsm.my.site.com/hsmonboarding/s/login/</t>
-  </si>
-  <si>
-    <t>HSM_Credential</t>
-  </si>
-  <si>
     <t>DestinationPath</t>
   </si>
   <si>
@@ -277,6 +281,18 @@
   </si>
   <si>
     <t>C:\Users\AnkushMyadam\Documents\MASTER DATA TEAM\GPO Portal\Hilton</t>
+  </si>
+  <si>
+    <t>https://suppliers.aramark-avendragroup.com/</t>
+  </si>
+  <si>
+    <t>Avendra_URL</t>
+  </si>
+  <si>
+    <t>Avendra_Credentials</t>
+  </si>
+  <si>
+    <t>Avendra_Credential</t>
   </si>
 </sst>
 </file>
@@ -364,9 +380,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -404,7 +420,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -510,7 +526,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -652,7 +668,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -661,12 +677,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="81.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -714,7 +730,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.5">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -724,7 +740,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="29">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1738,12 +1754,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z985"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="2" width="72.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="72.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1780,7 +1796,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="29">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1791,7 +1807,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.5">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -1905,7 +1921,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="29">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -1919,89 +1935,89 @@
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B31">
         <v>400</v>
@@ -2009,35 +2025,35 @@
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1"/>
@@ -2998,13 +3014,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="4" width="72.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="60.26953125" customWidth="1"/>
+    <col min="4" max="4" width="72.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3045,69 +3061,69 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
         <v>76</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" t="s">
         <v>77</v>
-      </c>
-      <c r="B7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>